<commit_message>
data: sync latest ADV drive sheets and submodule pointers
</commit_message>
<xml_diff>
--- a/res/drive/text assets/pevent/adv_pevent_003_ssmk_activity_021.xlsx
+++ b/res/drive/text assets/pevent/adv_pevent_003_ssmk_activity_021.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,14 @@
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -67,13 +75,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,27 +459,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>translated name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>translated text</t>
         </is>
@@ -491,7 +502,7 @@
 周りに星座のマークがついてるけど。</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>응? P치, 이 둥근 거 뭐야?
 주위에 별자리 마크가 붙어 있는데.</t>
@@ -515,7 +526,7 @@
 おみくじと番号占いが一度にできます。</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>확실히, 룰렛식 오미쿠지 기계입니다.
 오미쿠지와 번호 운세를 한 번에 할 수 있어요.</t>
@@ -539,7 +550,7 @@
 設置されていたらしいですよ。</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>옛날엔 여러 음식점에,
 설치되어 있었던 것 같아요.</t>
@@ -563,7 +574,7 @@
 ちょっとやってみよっかな！</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>와, 재밌겠다.
 나도 한번 해볼까!</t>
@@ -586,7 +597,7 @@
           <t>……あ、なんか出てきたよ！</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>……아, 뭔가 나왔네!</t>
         </is>
@@ -603,7 +614,7 @@
           <t>ピンクの紙ですね</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>분홍 종이네요</t>
         </is>
@@ -620,7 +631,7 @@
           <t>白い紙ですね</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>흰 종이네요</t>
         </is>
@@ -637,7 +648,7 @@
           <t>青い紙ですね</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>파란 종이네요</t>
         </is>
@@ -660,7 +671,7 @@
 おみくじは……やった、大吉ゲット♪</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>아, 운세 결과가 적혀 있어.
 오미쿠지는…… 좋았어, 대길 획득♪</t>
@@ -684,7 +695,7 @@
 嬉しいサプライズあり、だって。</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>번호 운세 쪽은……
 기쁜 서프라이즈가 있대.</t>
@@ -707,7 +718,7 @@
           <t>……っ！？</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>(……!?)</t>
         </is>
@@ -730,7 +741,7 @@
 なんかサプライズ用意してる感じ？</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>……P치, 혹시
 뭔가 서프라이즈 준비하고 있는 느낌?</t>
@@ -754,7 +765,7 @@
 楽しみだなぁ～♪</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>있잖아, 앞으로 뭐가 있는 거야～?
 기대된다～♪</t>
@@ -778,7 +789,7 @@
 おみくじは……中吉かぁ。</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>아, 운세 결과가 적혀 있어.
 오미쿠지는…… 중길이네.</t>
@@ -802,7 +813,7 @@
 今が伸び盛り、だって！</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>번호 운세 쪽은……
 지금이 한창 성장할 때래!</t>
@@ -825,7 +836,7 @@
           <t>レッスン、増やした方がいいかな？</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>레슨, 늘리는 게 좋을까?</t>
         </is>
@@ -848,9 +859,9 @@
 こちらが驚くぐらい成長していますよ。</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>세이카 씨는 이미 충분히 열심히 하고 있고,
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>스미카 씨는 이미 충분히 열심히 하고 있고,
 이쪽이 놀랄 정도로 성장하고 있어요.</t>
         </is>
       </c>
@@ -872,7 +883,7 @@
 へへっ、ありがと♪</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>……그럴까?
 헤헷, 고마워♪</t>
@@ -896,7 +907,7 @@
 おみくじは……うわ、凶だぁ……</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>아, 운세 결과가 적혀 있어.
 오미쿠지는…… 어, 흉이다……</t>
@@ -920,7 +931,7 @@
 本日アクシデントに注意、だって。</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>번호 운세 쪽은……
 오늘의 사고에 주의래.</t>
@@ -944,7 +955,7 @@
 今日は可能な限り、そばにいます。</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>……운세라지만 걱정되네요.
 오늘은 가능한 한 곁에 있겠습니다.</t>
@@ -967,7 +978,7 @@
           <t>……え、ほ、ほんとに！？</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>……에, 정, 정말!?</t>
         </is>
@@ -990,7 +1001,7 @@
 　ちょっと嬉しいかも♪）</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>(……운세는 좋지 않았지만,
 조금 기쁠지도♪)</t>

</xml_diff>